<commit_message>
feat(dashboard): split Signal Performance W/L into High/Close, relabel Prev as Open
Signal List Performance table now shows separate W/L columns for the
next-session High and Close vs the reference price (still the signal
session's close, now labelled "Open" in the UI/Excel export instead of
"Prev"). Migrates existing signal_results.csv + regenerates the daily
CSV/Excel review files to the new wl_high/wl_close schema.
</commit_message>
<xml_diff>
--- a/data/performance/daily/signal_list_2026-05-12.xlsx
+++ b/data/performance/daily/signal_list_2026-05-12.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Swing" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Scalping" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swing" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scalping" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:K125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -461,9 +461,10 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,7 +494,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -518,15 +519,20 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>W/L</t>
+          <t>W/L High</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
+          <t>W/L Close</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
           <t>Eval Date</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -563,12 +569,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -600,17 +611,22 @@
       <c r="G6" s="4" t="n">
         <v>-0.98</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -642,17 +658,22 @@
       <c r="G7" s="4" t="n">
         <v>-0.39</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -684,17 +705,22 @@
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -726,17 +752,22 @@
       <c r="G9" s="4" t="n">
         <v>-6.6</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -773,12 +804,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -810,17 +846,22 @@
       <c r="G11" s="4" t="n">
         <v>-0.84</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -852,17 +893,22 @@
       <c r="G12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -899,12 +945,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -941,12 +992,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -983,12 +1039,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1025,12 +1086,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1062,17 +1128,22 @@
       <c r="G17" s="4" t="n">
         <v>-0.72</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1104,17 +1175,22 @@
       <c r="G18" s="4" t="n">
         <v>-3.03</v>
       </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1146,17 +1222,22 @@
       <c r="G19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1188,17 +1269,22 @@
       <c r="G20" s="4" t="n">
         <v>-0.5</v>
       </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1235,12 +1321,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1277,12 +1368,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1314,17 +1410,22 @@
       <c r="G23" s="4" t="n">
         <v>-6.43</v>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1356,17 +1457,22 @@
       <c r="G24" s="4" t="n">
         <v>-0.22</v>
       </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1398,17 +1504,22 @@
       <c r="G25" s="4" t="n">
         <v>-2.96</v>
       </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1440,17 +1551,22 @@
       <c r="G26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1482,17 +1598,22 @@
       <c r="G27" s="4" t="n">
         <v>-7.11</v>
       </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1529,12 +1650,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1566,17 +1692,22 @@
       <c r="G29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1613,12 +1744,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1655,12 +1791,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1697,12 +1838,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1734,17 +1880,22 @@
       <c r="G33" s="4" t="n">
         <v>-0.66</v>
       </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1776,17 +1927,22 @@
       <c r="G34" s="4" t="n">
         <v>-5.93</v>
       </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1818,17 +1974,22 @@
       <c r="G35" s="4" t="n">
         <v>-2.33</v>
       </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1860,17 +2021,22 @@
       <c r="G36" s="4" t="n">
         <v>-3</v>
       </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1902,17 +2068,22 @@
       <c r="G37" s="4" t="n">
         <v>-2.94</v>
       </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1944,17 +2115,22 @@
       <c r="G38" s="4" t="n">
         <v>-10.24</v>
       </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1986,17 +2162,22 @@
       <c r="G39" s="4" t="n">
         <v>-0.57</v>
       </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2033,12 +2214,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2070,17 +2256,22 @@
       <c r="G41" s="4" t="n">
         <v>-3.62</v>
       </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2117,12 +2308,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2159,12 +2355,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2196,17 +2397,22 @@
       <c r="G44" s="4" t="n">
         <v>-1.98</v>
       </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2238,17 +2444,22 @@
       <c r="G45" s="4" t="n">
         <v>-5.65</v>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2280,17 +2491,22 @@
       <c r="G46" s="4" t="n">
         <v>-2.33</v>
       </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2327,12 +2543,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2364,17 +2585,22 @@
       <c r="G48" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2406,17 +2632,22 @@
       <c r="G49" s="4" t="n">
         <v>-8.550000000000001</v>
       </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2453,12 +2684,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2495,12 +2731,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2537,12 +2778,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2579,12 +2825,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2621,12 +2872,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2663,12 +2919,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2700,17 +2961,22 @@
       <c r="G56" s="4" t="n">
         <v>-4.55</v>
       </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2747,12 +3013,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2784,17 +3055,22 @@
       <c r="G58" s="4" t="n">
         <v>-1.15</v>
       </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2826,17 +3102,22 @@
       <c r="G59" s="4" t="n">
         <v>-6.99</v>
       </c>
-      <c r="H59" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2868,17 +3149,22 @@
       <c r="G60" s="4" t="n">
         <v>-14.55</v>
       </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2915,12 +3201,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2952,17 +3243,22 @@
       <c r="G62" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2994,17 +3290,22 @@
       <c r="G63" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3036,17 +3337,22 @@
       <c r="G64" s="4" t="n">
         <v>-9.09</v>
       </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3083,12 +3389,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3125,12 +3436,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3162,17 +3478,22 @@
       <c r="G67" s="4" t="n">
         <v>-1.2</v>
       </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3204,17 +3525,22 @@
       <c r="G68" s="4" t="n">
         <v>-5.62</v>
       </c>
-      <c r="H68" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3246,17 +3572,22 @@
       <c r="G69" s="4" t="n">
         <v>-2.17</v>
       </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3288,17 +3619,22 @@
       <c r="G70" s="4" t="n">
         <v>-2.87</v>
       </c>
-      <c r="H70" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3330,17 +3666,22 @@
       <c r="G71" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3372,17 +3713,22 @@
       <c r="G72" s="4" t="n">
         <v>-14.58</v>
       </c>
-      <c r="H72" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3419,12 +3765,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3461,12 +3812,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3498,17 +3854,22 @@
       <c r="G75" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3540,17 +3901,22 @@
       <c r="G76" s="4" t="n">
         <v>-7.29</v>
       </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3582,17 +3948,22 @@
       <c r="G77" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3624,17 +3995,22 @@
       <c r="G78" s="4" t="n">
         <v>-9.32</v>
       </c>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3671,12 +4047,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3713,12 +4094,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3750,17 +4136,22 @@
       <c r="G81" s="4" t="n">
         <v>-7.94</v>
       </c>
-      <c r="H81" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3797,12 +4188,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3839,12 +4235,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3876,17 +4277,22 @@
       <c r="G84" s="4" t="n">
         <v>-8.93</v>
       </c>
-      <c r="H84" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3923,12 +4329,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -3965,12 +4376,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4002,17 +4418,22 @@
       <c r="G87" s="4" t="n">
         <v>-0.88</v>
       </c>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4044,17 +4465,22 @@
       <c r="G88" s="4" t="n">
         <v>-4.83</v>
       </c>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4086,17 +4512,22 @@
       <c r="G89" s="4" t="n">
         <v>-4.76</v>
       </c>
-      <c r="H89" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4133,12 +4564,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4175,12 +4611,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4217,12 +4658,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4254,17 +4700,22 @@
       <c r="G93" s="4" t="n">
         <v>-2.63</v>
       </c>
-      <c r="H93" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4296,17 +4747,22 @@
       <c r="G94" s="4" t="n">
         <v>-1.22</v>
       </c>
-      <c r="H94" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4343,12 +4799,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4380,17 +4841,22 @@
       <c r="G96" s="4" t="n">
         <v>-8.33</v>
       </c>
-      <c r="H96" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4427,12 +4893,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4469,12 +4940,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4506,17 +4982,22 @@
       <c r="G99" s="4" t="n">
         <v>-10.34</v>
       </c>
-      <c r="H99" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4548,17 +5029,22 @@
       <c r="G100" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H100" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4590,17 +5076,22 @@
       <c r="G101" s="4" t="n">
         <v>-13.4</v>
       </c>
-      <c r="H101" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4637,12 +5128,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4674,17 +5170,22 @@
       <c r="G103" s="4" t="n">
         <v>-1.55</v>
       </c>
-      <c r="H103" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4716,17 +5217,22 @@
       <c r="G104" s="4" t="n">
         <v>-2.33</v>
       </c>
-      <c r="H104" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I104" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4758,17 +5264,22 @@
       <c r="G105" s="4" t="n">
         <v>-4.07</v>
       </c>
-      <c r="H105" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4805,12 +5316,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4842,17 +5358,22 @@
       <c r="G107" s="4" t="n">
         <v>-11.7</v>
       </c>
-      <c r="H107" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4884,17 +5405,22 @@
       <c r="G108" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H108" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4926,17 +5452,22 @@
       <c r="G109" s="4" t="n">
         <v>-1.9</v>
       </c>
-      <c r="H109" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -4968,17 +5499,22 @@
       <c r="G110" s="4" t="n">
         <v>-14.81</v>
       </c>
-      <c r="H110" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5010,17 +5546,22 @@
       <c r="G111" s="4" t="n">
         <v>-1.96</v>
       </c>
-      <c r="H111" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5052,17 +5593,22 @@
       <c r="G112" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H112" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I112" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5094,17 +5640,22 @@
       <c r="G113" s="4" t="n">
         <v>-11.26</v>
       </c>
-      <c r="H113" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I113" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5136,17 +5687,22 @@
       <c r="G114" s="4" t="n">
         <v>-0.83</v>
       </c>
-      <c r="H114" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5183,12 +5739,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I115" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5220,17 +5781,22 @@
       <c r="G116" s="4" t="n">
         <v>-6.67</v>
       </c>
-      <c r="H116" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I116" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5262,17 +5828,22 @@
       <c r="G117" s="4" t="n">
         <v>-12.36</v>
       </c>
-      <c r="H117" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I117" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5309,12 +5880,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I118" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5351,12 +5927,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5393,12 +5974,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I120" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5430,17 +6016,22 @@
       <c r="G121" s="4" t="n">
         <v>-12.23</v>
       </c>
-      <c r="H121" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H121" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I121" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5472,17 +6063,22 @@
       <c r="G122" s="4" t="n">
         <v>-1.92</v>
       </c>
-      <c r="H122" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5514,17 +6110,22 @@
       <c r="G123" s="4" t="n">
         <v>-7.14</v>
       </c>
-      <c r="H123" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="I123" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5561,12 +6162,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I124" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5603,12 +6209,17 @@
           <t>W</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
+      <c r="I125" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -5625,7 +6236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5635,9 +6246,10 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5667,7 +6279,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -5692,15 +6304,20 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>W/L</t>
+          <t>W/L High</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
+          <t>W/L Close</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
           <t>Eval Date</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>